<commit_message>
n8n board refresh 2026-06-27T17:38:10Z
</commit_message>
<xml_diff>
--- a/app/reports/HCA_research.xlsx
+++ b/app/reports/HCA_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-26 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-27 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>391.4225</v>
+        <v>391.68</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.297</v>
+        <v>0.296</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>0.797</v>
+        <v>0.796</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04372000217437744</v>
+        <v>0.04372</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>221839793.2259898</v>
+        <v>221839811.7647059</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>391.4225</v>
+        <v>391.68</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>86833086464</v>
+        <v>86890217472</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>13.49</v>
+        <v>13.5</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>8.859999999999999</v>
+        <v>8.93</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.81</v>
+        <v>1.82</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>116275535872</v>
+        <v>117459943424</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>15.94958</v>
+        <v>16.112045</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>7.857</v>
+        <v>8.087</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>3.075</v>
+        <v>3.165</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>133570445312</v>
+        <v>133130248192</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>45.914474</v>
+        <v>45.563316</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>12.994</v>
+        <v>12.967</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>0.494</v>
+        <v>0.493</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>104603361280</v>
+        <v>105174310912</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>13.924</v>
+        <v>14.037433</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>10.456</v>
+        <v>10.563</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>3.647</v>
+        <v>3.684</v>
       </c>
     </row>
     <row r="9">
@@ -1616,13 +1616,13 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>90251132928</v>
+        <v>89390030848</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>20.106024</v>
+        <v>19.883072</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>14.23</v>
+        <v>14.225</v>
       </c>
       <c r="F9" s="34" t="n">
         <v>0.243</v>
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>103568457728</v>
+        <v>103658061824</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>21.69169</v>
+        <v>21.710457</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>12.235</v>
+        <v>12.293</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>3.399</v>
+        <v>3.415</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>137356607488</v>
+        <v>138439507968</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>18.396948</v>
+        <v>18.541986</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>7.339</v>
+        <v>7.478</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>2.951</v>
+        <v>3.007</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>101866840064</v>
+        <v>102812377088</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>18.913334</v>
+        <v>19.08889</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>9.003</v>
+        <v>9.218999999999999</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>2.439</v>
+        <v>2.497</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>126585733120</v>
+        <v>127547957248</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>38.26188</v>
+        <v>38.463585</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>19.291</v>
+        <v>20.211</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>5.281</v>
+        <v>5.533</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-06-28T17:37:47Z
</commit_message>
<xml_diff>
--- a/app/reports/HCA_research.xlsx
+++ b/app/reports/HCA_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-27 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-28 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04372</v>
+        <v>0.04372000217437744</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
n8n board refresh 2026-06-29T17:39:52Z
</commit_message>
<xml_diff>
--- a/app/reports/HCA_research.xlsx
+++ b/app/reports/HCA_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-28 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-29 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>507.78</v>
+        <v>507.32</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>391.68</v>
+        <v>391.15</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.296</v>
+        <v>0.297</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>0.796</v>
+        <v>0.797</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04372000217437744</v>
+        <v>0.04375999927520752</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>221839811.7647059</v>
+        <v>221839799.8108143</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>391.68</v>
+        <v>391.15</v>
       </c>
     </row>
     <row r="38">
@@ -1520,10 +1520,10 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>86890217472</v>
+        <v>86772637696</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>13.5</v>
+        <v>13.48</v>
       </c>
       <c r="E5" s="32" t="n">
         <v>8.93</v>
@@ -1544,10 +1544,10 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>117459943424</v>
+        <v>117837725696</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>16.112045</v>
+        <v>16.163866</v>
       </c>
       <c r="E6" s="34" t="n">
         <v>8.087</v>
@@ -1568,10 +1568,10 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>133130248192</v>
+        <v>132345552896</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>45.563316</v>
+        <v>45.29476</v>
       </c>
       <c r="E7" s="34" t="n">
         <v>12.967</v>
@@ -1592,10 +1592,10 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>105174310912</v>
+        <v>105054109696</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>14.037433</v>
+        <v>14.02139</v>
       </c>
       <c r="E8" s="34" t="n">
         <v>10.563</v>
@@ -1616,10 +1616,10 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>89390030848</v>
+        <v>88123244544</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>19.883072</v>
+        <v>19.601301</v>
       </c>
       <c r="E9" s="34" t="n">
         <v>14.225</v>
@@ -1640,10 +1640,10 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>103658061824</v>
+        <v>104118870016</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>21.710457</v>
+        <v>21.806969</v>
       </c>
       <c r="E10" s="34" t="n">
         <v>12.293</v>
@@ -1664,10 +1664,10 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>138439507968</v>
+        <v>138012049408</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>18.541986</v>
+        <v>18.484734</v>
       </c>
       <c r="E11" s="34" t="n">
         <v>7.478</v>
@@ -1688,10 +1688,10 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>102812377088</v>
+        <v>103183409152</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>19.08889</v>
+        <v>19.157778</v>
       </c>
       <c r="E12" s="34" t="n">
         <v>9.218999999999999</v>
@@ -1712,10 +1712,10 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>127547957248</v>
+        <v>127915991040</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>38.463585</v>
+        <v>38.57457</v>
       </c>
       <c r="E13" s="34" t="n">
         <v>20.211</v>

</xml_diff>

<commit_message>
n8n board refresh 2026-06-30T17:38:51Z
</commit_message>
<xml_diff>
--- a/app/reports/HCA_research.xlsx
+++ b/app/reports/HCA_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-29 17:36 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-30 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.83</v>
+        <v>0.829</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>507.32</v>
+        <v>503.47</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>391.15</v>
+        <v>388.705</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.297</v>
+        <v>0.295</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>0.797</v>
+        <v>0.795</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04375999927520752</v>
+        <v>0.04409999847412109</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>221839799.8108143</v>
+        <v>221839794.1472325</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>391.15</v>
+        <v>388.705</v>
       </c>
     </row>
     <row r="38">
@@ -1520,13 +1520,13 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>86772637696</v>
+        <v>86230237184</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>13.48</v>
+        <v>13.39</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>8.93</v>
+        <v>8.94</v>
       </c>
       <c r="F5" s="32" t="n">
         <v>1.82</v>
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>117837725696</v>
+        <v>118338035712</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>16.163866</v>
+        <v>16.232494</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>8.087</v>
+        <v>8.199</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>3.165</v>
+        <v>3.209</v>
       </c>
     </row>
     <row r="7">
@@ -1568,16 +1568,16 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>132345552896</v>
+        <v>132428496896</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>45.29476</v>
+        <v>45.52193</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>12.967</v>
+        <v>12.905</v>
       </c>
       <c r="F7" s="34" t="n">
-        <v>0.493</v>
+        <v>0.49</v>
       </c>
     </row>
     <row r="8">
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>105054109696</v>
+        <v>105194340352</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>14.02139</v>
+        <v>14.002666</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>10.563</v>
+        <v>10.617</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>3.684</v>
+        <v>3.703</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>88123244544</v>
+        <v>88020803584</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>19.601301</v>
+        <v>19.604042</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>14.225</v>
+        <v>13.946</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>0.243</v>
+        <v>0.238</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>104118870016</v>
+        <v>101046771712</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>21.806969</v>
+        <v>21.16354</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>12.293</v>
+        <v>12.287</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>3.415</v>
+        <v>3.414</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>138012049408</v>
+        <v>137556082688</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>18.484734</v>
+        <v>18.423666</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>7.478</v>
+        <v>7.496</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>3.007</v>
+        <v>3.014</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>103183409152</v>
+        <v>102596935680</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>19.157778</v>
+        <v>19.04889</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>9.218999999999999</v>
+        <v>9.308999999999999</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>2.497</v>
+        <v>2.522</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>127915991040</v>
+        <v>119963164672</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>38.57457</v>
+        <v>36.260136</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>20.211</v>
+        <v>20.089</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>5.533</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
n8n board refresh 2026-07-01T17:40:12Z
</commit_message>
<xml_diff>
--- a/app/reports/HCA_research.xlsx
+++ b/app/reports/HCA_research.xlsx
@@ -621,7 +621,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-30 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-07-01 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.829</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>503.47</v>
+        <v>497.1</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>388.705</v>
+        <v>391.985</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>0.295</v>
+        <v>0.268</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>0.795</v>
+        <v>0.768</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>0.04409999847412109</v>
+        <v>0.04467000007629394</v>
       </c>
     </row>
     <row r="6">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B35" s="21" t="n">
-        <v>221839794.1472325</v>
+        <v>221839803.0536883</v>
       </c>
     </row>
     <row r="36">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="B37" s="23" t="n">
-        <v>388.705</v>
+        <v>391.985</v>
       </c>
     </row>
     <row r="38">
@@ -1520,16 +1520,16 @@
         </is>
       </c>
       <c r="C5" s="31" t="n">
-        <v>86230237184</v>
+        <v>86957875200</v>
       </c>
       <c r="D5" s="32" t="n">
-        <v>13.39</v>
+        <v>13.49</v>
       </c>
       <c r="E5" s="32" t="n">
-        <v>8.94</v>
+        <v>8.9</v>
       </c>
       <c r="F5" s="32" t="n">
-        <v>1.82</v>
+        <v>1.81</v>
       </c>
     </row>
     <row r="6">
@@ -1544,16 +1544,16 @@
         </is>
       </c>
       <c r="C6" s="33" t="n">
-        <v>118338035712</v>
+        <v>115315769344</v>
       </c>
       <c r="D6" s="34" t="n">
-        <v>16.232494</v>
+        <v>15.817927</v>
       </c>
       <c r="E6" s="34" t="n">
-        <v>8.199</v>
+        <v>8.097</v>
       </c>
       <c r="F6" s="34" t="n">
-        <v>3.209</v>
+        <v>3.169</v>
       </c>
     </row>
     <row r="7">
@@ -1568,13 +1568,13 @@
         </is>
       </c>
       <c r="C7" s="33" t="n">
-        <v>132428496896</v>
+        <v>133319467008</v>
       </c>
       <c r="D7" s="34" t="n">
-        <v>45.52193</v>
+        <v>45.8282</v>
       </c>
       <c r="E7" s="34" t="n">
-        <v>12.905</v>
+        <v>12.894</v>
       </c>
       <c r="F7" s="34" t="n">
         <v>0.49</v>
@@ -1592,16 +1592,16 @@
         </is>
       </c>
       <c r="C8" s="33" t="n">
-        <v>105194340352</v>
+        <v>102413058048</v>
       </c>
       <c r="D8" s="34" t="n">
-        <v>14.002666</v>
+        <v>13.636</v>
       </c>
       <c r="E8" s="34" t="n">
-        <v>10.617</v>
+        <v>10.549</v>
       </c>
       <c r="F8" s="34" t="n">
-        <v>3.703</v>
+        <v>3.679</v>
       </c>
     </row>
     <row r="9">
@@ -1616,16 +1616,16 @@
         </is>
       </c>
       <c r="C9" s="33" t="n">
-        <v>88020803584</v>
+        <v>89853648896</v>
       </c>
       <c r="D9" s="34" t="n">
-        <v>19.604042</v>
+        <v>19.99661</v>
       </c>
       <c r="E9" s="34" t="n">
-        <v>13.946</v>
+        <v>14.087</v>
       </c>
       <c r="F9" s="34" t="n">
-        <v>0.238</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="10">
@@ -1640,16 +1640,16 @@
         </is>
       </c>
       <c r="C10" s="33" t="n">
-        <v>101046771712</v>
+        <v>101353979904</v>
       </c>
       <c r="D10" s="34" t="n">
-        <v>21.16354</v>
+        <v>21.227882</v>
       </c>
       <c r="E10" s="34" t="n">
-        <v>12.287</v>
+        <v>11.945</v>
       </c>
       <c r="F10" s="34" t="n">
-        <v>3.414</v>
+        <v>3.319</v>
       </c>
     </row>
     <row r="11">
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>137556082688</v>
+        <v>135903240192</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>18.423666</v>
+        <v>18.20229</v>
       </c>
       <c r="E11" s="34" t="n">
-        <v>7.496</v>
+        <v>7.431</v>
       </c>
       <c r="F11" s="34" t="n">
-        <v>3.014</v>
+        <v>2.988</v>
       </c>
     </row>
     <row r="12">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="C12" s="33" t="n">
-        <v>102596935680</v>
+        <v>98970378240</v>
       </c>
       <c r="D12" s="34" t="n">
-        <v>19.04889</v>
+        <v>18.294249</v>
       </c>
       <c r="E12" s="34" t="n">
-        <v>9.308999999999999</v>
+        <v>9.164999999999999</v>
       </c>
       <c r="F12" s="34" t="n">
-        <v>2.522</v>
+        <v>2.482</v>
       </c>
     </row>
     <row r="13">
@@ -1712,16 +1712,16 @@
         </is>
       </c>
       <c r="C13" s="33" t="n">
-        <v>119963164672</v>
+        <v>119545298944</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>36.260136</v>
+        <v>36.133835</v>
       </c>
       <c r="E13" s="34" t="n">
-        <v>20.089</v>
+        <v>19.22</v>
       </c>
       <c r="F13" s="34" t="n">
-        <v>5.5</v>
+        <v>5.262</v>
       </c>
     </row>
     <row r="15">

</xml_diff>